<commit_message>
Add a second empty week block (J:K) to the Open WOs tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016Ld5yLC3t3yCVGVfyBR5pc
</commit_message>
<xml_diff>
--- a/open-wos-weekly-tracker/Open_WOs_tracker.xlsx
+++ b/open-wos-weekly-tracker/Open_WOs_tracker.xlsx
@@ -1951,7 +1951,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D133B0A-06FD-4F6C-BECC-32CA9848D96D}">
   <sheetPr/>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="3" customWidth="1"/>
@@ -2064,6 +2064,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="8"/>
+      <c r="J1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="K1" s="8"/>
     </row>
     <row r="2" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A2" s="16"/>
@@ -2072,6 +2076,8 @@
       <c r="E2" s="17"/>
       <c r="G2" s="16"/>
       <c r="H2" s="17"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="17"/>
     </row>
     <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="42" t="s">
@@ -2086,6 +2092,10 @@
         <v>1</v>
       </c>
       <c r="H3" s="42"/>
+      <c r="J3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3" s="42"/>
     </row>
     <row r="4" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
@@ -2104,6 +2114,10 @@
       <c r="H4" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="J4" s="5"/>
+      <c r="K4" s="6" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="5" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
@@ -2120,6 +2134,10 @@
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="5"/>
+      <c r="K5" s="6" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2145,6 +2163,13 @@
       <c r="H6" s="6" t="s">
         <v>4</v>
       </c>
+      <c r="J6" s="5">
+        <f>SUM(J4+J5)</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="7" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
@@ -2162,6 +2187,10 @@
         <v>5</v>
       </c>
       <c r="H8" s="43"/>
+      <c r="J8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="K8" s="43"/>
     </row>
     <row r="9" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
@@ -2180,6 +2209,10 @@
       <c r="H9" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="J9" s="5"/>
+      <c r="K9" s="6" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
@@ -2196,6 +2229,10 @@
       </c>
       <c r="G10" s="5"/>
       <c r="H10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="J10" s="5"/>
+      <c r="K10" s="6" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2221,6 +2258,13 @@
       <c r="H11" s="6" t="s">
         <v>4</v>
       </c>
+      <c r="J11" s="5">
+        <f>SUM(J9+J10)</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="12" x14ac:dyDescent="0.25">
       <c r="D12" s="3"/>
@@ -2238,6 +2282,10 @@
         <v>6</v>
       </c>
       <c r="H13" s="44"/>
+      <c r="J13" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="K13" s="44"/>
     </row>
     <row r="14" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
@@ -2259,6 +2307,13 @@
         <v>0</v>
       </c>
       <c r="H14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J14" s="5">
+        <f>SUM(J6+J11)</f>
+        <v>0</v>
+      </c>
+      <c r="K14" s="6" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2275,12 +2330,12 @@
     <row r="17">
       <c r="A17" s="31" t="inlineStr">
         <is>
-          <t>Next week: copy the newest block (for example G1:H14), paste it 3 columns to the right (J1), and fill in the yellow cells. The chart on Sheet1 updates by itself.</t>
+          <t>When the empty blocks are used up: copy the newest block (for example J1:K14), paste it 3 columns to the right (M1), and fill in the yellow cells. The chart on Sheet1 updates by itself.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="12">
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A13:B13"/>
@@ -2290,6 +2345,9 @@
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="G13:H13"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="J13:K13"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:ZZ1">
     <cfRule type="expression" dxfId="18" priority="1">

</xml_diff>

<commit_message>
Add a third empty week block (M:N) to the Open WOs tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016Ld5yLC3t3yCVGVfyBR5pc
</commit_message>
<xml_diff>
--- a/open-wos-weekly-tracker/Open_WOs_tracker.xlsx
+++ b/open-wos-weekly-tracker/Open_WOs_tracker.xlsx
@@ -1951,7 +1951,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D133B0A-06FD-4F6C-BECC-32CA9848D96D}">
   <sheetPr/>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="3" customWidth="1"/>
@@ -2068,6 +2068,10 @@
         <v>0</v>
       </c>
       <c r="K1" s="8"/>
+      <c r="M1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="8"/>
     </row>
     <row r="2" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A2" s="16"/>
@@ -2078,6 +2082,8 @@
       <c r="H2" s="17"/>
       <c r="J2" s="16"/>
       <c r="K2" s="17"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="17"/>
     </row>
     <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="42" t="s">
@@ -2096,6 +2102,10 @@
         <v>1</v>
       </c>
       <c r="K3" s="42"/>
+      <c r="M3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="N3" s="42"/>
     </row>
     <row r="4" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
@@ -2118,6 +2128,10 @@
       <c r="K4" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="M4" s="5"/>
+      <c r="N4" s="6" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="5" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
@@ -2138,6 +2152,10 @@
       </c>
       <c r="J5" s="5"/>
       <c r="K5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="M5" s="5"/>
+      <c r="N5" s="6" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2170,6 +2188,13 @@
       <c r="K6" s="6" t="s">
         <v>4</v>
       </c>
+      <c r="M6" s="5">
+        <f>SUM(M4+M5)</f>
+        <v>0</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="7" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
@@ -2191,6 +2216,10 @@
         <v>5</v>
       </c>
       <c r="K8" s="43"/>
+      <c r="M8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="N8" s="43"/>
     </row>
     <row r="9" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
@@ -2213,6 +2242,10 @@
       <c r="K9" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="M9" s="5"/>
+      <c r="N9" s="6" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
@@ -2233,6 +2266,10 @@
       </c>
       <c r="J10" s="5"/>
       <c r="K10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="M10" s="5"/>
+      <c r="N10" s="6" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2265,6 +2302,13 @@
       <c r="K11" s="6" t="s">
         <v>4</v>
       </c>
+      <c r="M11" s="5">
+        <f>SUM(M9+M10)</f>
+        <v>0</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="12" x14ac:dyDescent="0.25">
       <c r="D12" s="3"/>
@@ -2286,6 +2330,10 @@
         <v>6</v>
       </c>
       <c r="K13" s="44"/>
+      <c r="M13" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="N13" s="44"/>
     </row>
     <row r="14" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
@@ -2314,6 +2362,13 @@
         <v>0</v>
       </c>
       <c r="K14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M14" s="5">
+        <f>SUM(M6+M11)</f>
+        <v>0</v>
+      </c>
+      <c r="N14" s="6" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2330,12 +2385,12 @@
     <row r="17">
       <c r="A17" s="31" t="inlineStr">
         <is>
-          <t>When the empty blocks are used up: copy the newest block (for example J1:K14), paste it 3 columns to the right (M1), and fill in the yellow cells. The chart on Sheet1 updates by itself.</t>
+          <t>When the empty blocks are used up: copy the newest block (for example M1:N14), paste it 3 columns to the right (P1), and fill in the yellow cells. The chart on Sheet1 updates by itself.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="15">
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A13:B13"/>
@@ -2348,6 +2403,9 @@
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="J8:K8"/>
     <mergeCell ref="J13:K13"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="M13:N13"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:ZZ1">
     <cfRule type="expression" dxfId="18" priority="1">

</xml_diff>

<commit_message>
Pre-build weekly blocks through end of 2026 in the Open WOs tracker
One dated block per Monday from 9/28 to 12/28. The table on Sheet1 now
counts a block only when it has a date and at least one number, so the
empty future blocks stay off the chart.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016Ld5yLC3t3yCVGVfyBR5pc
</commit_message>
<xml_diff>
--- a/open-wos-weekly-tracker/Open_WOs_tracker.xlsx
+++ b/open-wos-weekly-tracker/Open_WOs_tracker.xlsx
@@ -1608,8 +1608,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FAA67808-CB3C-417B-9344-CB465344E1E7}" name="WeeklyLog" displayName="WeeklyLog" ref="A21:I47" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
-  <autoFilter ref="A21:I47" xr:uid="{FAA67808-CB3C-417B-9344-CB465344E1E7}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FAA67808-CB3C-417B-9344-CB465344E1E7}" name="WeeklyLog" displayName="WeeklyLog" ref="A21:I61" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+  <autoFilter ref="A21:I61" xr:uid="{FAA67808-CB3C-417B-9344-CB465344E1E7}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1622,22 +1622,22 @@
   </autoFilter>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{C147C25E-F3F6-4B45-B9D8-E6FCD9403FCD}" name="Week Of" dataDxfId="8">
-      <calculatedColumnFormula>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</calculatedColumnFormula>
+      <calculatedColumnFormula>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{D5CF7A79-7DDD-4B83-8875-CCD6C8D9E42D}" name="Burnsville Repair Tickets" dataDxfId="7">
-      <calculatedColumnFormula>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</calculatedColumnFormula>
+      <calculatedColumnFormula>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{C49CEAF5-521E-4B6D-9855-C9264B51FF10}" name="Burnsville PMs" dataDxfId="6">
-      <calculatedColumnFormula>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</calculatedColumnFormula>
+      <calculatedColumnFormula>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{DEEE7B5D-DDBA-4E11-85BC-C3DC53551764}" name="Burnsville Total" dataDxfId="5">
       <calculatedColumnFormula>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{87460474-A791-4B36-9A6A-38F4E93B1F7B}" name="Lakeville Repair Tickets" dataDxfId="4">
-      <calculatedColumnFormula>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</calculatedColumnFormula>
+      <calculatedColumnFormula>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{E558F3A5-D9CB-4C23-AA9F-7293BC7F900F}" name="Lakeville PMs" dataDxfId="3">
-      <calculatedColumnFormula>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</calculatedColumnFormula>
+      <calculatedColumnFormula>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{C1803D2A-0953-4951-86B5-83796D01D2E4}" name="Lakeville Total" dataDxfId="2">
       <calculatedColumnFormula>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</calculatedColumnFormula>
@@ -1951,7 +1951,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D133B0A-06FD-4F6C-BECC-32CA9848D96D}">
   <sheetPr/>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:AU17"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="3" customWidth="1"/>
@@ -2044,7 +2044,37 @@
     <col min="88" max="88" width="9.140625" style="4" customWidth="1"/>
     <col min="89" max="89" width="27" style="4" customWidth="1"/>
     <col min="90" max="90" width="9.140625" style="4" customWidth="1"/>
-    <col min="91" max="16384" width="9.140625" style="4"/>
+    <col min="91" max="91" width="9.140625" style="4" customWidth="1"/>
+    <col min="92" max="92" width="27" style="4" customWidth="1"/>
+    <col min="93" max="93" width="9.140625" style="4" customWidth="1"/>
+    <col min="94" max="94" width="9.140625" style="4" customWidth="1"/>
+    <col min="95" max="95" width="27" style="4" customWidth="1"/>
+    <col min="96" max="96" width="9.140625" style="4" customWidth="1"/>
+    <col min="97" max="97" width="9.140625" style="4" customWidth="1"/>
+    <col min="98" max="98" width="27" style="4" customWidth="1"/>
+    <col min="99" max="99" width="9.140625" style="4" customWidth="1"/>
+    <col min="100" max="100" width="9.140625" style="4" customWidth="1"/>
+    <col min="101" max="101" width="27" style="4" customWidth="1"/>
+    <col min="102" max="102" width="9.140625" style="4" customWidth="1"/>
+    <col min="103" max="103" width="9.140625" style="4" customWidth="1"/>
+    <col min="104" max="104" width="27" style="4" customWidth="1"/>
+    <col min="105" max="105" width="9.140625" style="4" customWidth="1"/>
+    <col min="106" max="106" width="9.140625" style="4" customWidth="1"/>
+    <col min="107" max="107" width="27" style="4" customWidth="1"/>
+    <col min="108" max="108" width="9.140625" style="4" customWidth="1"/>
+    <col min="109" max="109" width="9.140625" style="4" customWidth="1"/>
+    <col min="110" max="110" width="27" style="4" customWidth="1"/>
+    <col min="111" max="111" width="9.140625" style="4" customWidth="1"/>
+    <col min="112" max="112" width="9.140625" style="4" customWidth="1"/>
+    <col min="113" max="113" width="27" style="4" customWidth="1"/>
+    <col min="114" max="114" width="9.140625" style="4" customWidth="1"/>
+    <col min="115" max="115" width="9.140625" style="4" customWidth="1"/>
+    <col min="116" max="116" width="27" style="4" customWidth="1"/>
+    <col min="117" max="117" width="9.140625" style="4" customWidth="1"/>
+    <col min="118" max="118" width="9.140625" style="4" customWidth="1"/>
+    <col min="119" max="119" width="27" style="4" customWidth="1"/>
+    <col min="120" max="120" width="9.140625" style="4" customWidth="1"/>
+    <col min="121" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" x14ac:dyDescent="0.25">
@@ -2063,15 +2093,87 @@
       <c r="G1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="8"/>
+      <c r="H1" s="8">
+        <v>46293</v>
+      </c>
       <c r="J1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="K1" s="8"/>
+      <c r="K1" s="8">
+        <v>46300</v>
+      </c>
       <c r="M1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="N1" s="8"/>
+      <c r="N1" s="8">
+        <v>46307</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q1" s="8">
+        <v>46314</v>
+      </c>
+      <c r="S1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="T1" s="8">
+        <v>46321</v>
+      </c>
+      <c r="V1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="W1" s="8">
+        <v>46328</v>
+      </c>
+      <c r="Y1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="Z1" s="8">
+        <v>46335</v>
+      </c>
+      <c r="AB1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="AC1" s="8">
+        <v>46342</v>
+      </c>
+      <c r="AE1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF1" s="8">
+        <v>46349</v>
+      </c>
+      <c r="AH1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI1" s="8">
+        <v>46356</v>
+      </c>
+      <c r="AK1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="AL1" s="8">
+        <v>46363</v>
+      </c>
+      <c r="AN1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="AO1" s="8">
+        <v>46370</v>
+      </c>
+      <c r="AQ1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="AR1" s="8">
+        <v>46377</v>
+      </c>
+      <c r="AT1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="AU1" s="8">
+        <v>46384</v>
+      </c>
     </row>
     <row r="2" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A2" s="16"/>
@@ -2084,6 +2186,28 @@
       <c r="K2" s="17"/>
       <c r="M2" s="16"/>
       <c r="N2" s="17"/>
+      <c r="P2" s="16"/>
+      <c r="Q2" s="17"/>
+      <c r="S2" s="16"/>
+      <c r="T2" s="17"/>
+      <c r="V2" s="16"/>
+      <c r="W2" s="17"/>
+      <c r="Y2" s="16"/>
+      <c r="Z2" s="17"/>
+      <c r="AB2" s="16"/>
+      <c r="AC2" s="17"/>
+      <c r="AE2" s="16"/>
+      <c r="AF2" s="17"/>
+      <c r="AH2" s="16"/>
+      <c r="AI2" s="17"/>
+      <c r="AK2" s="16"/>
+      <c r="AL2" s="17"/>
+      <c r="AN2" s="16"/>
+      <c r="AO2" s="17"/>
+      <c r="AQ2" s="16"/>
+      <c r="AR2" s="17"/>
+      <c r="AT2" s="16"/>
+      <c r="AU2" s="17"/>
     </row>
     <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="42" t="s">
@@ -2106,6 +2230,50 @@
         <v>1</v>
       </c>
       <c r="N3" s="42"/>
+      <c r="P3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="42"/>
+      <c r="S3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="T3" s="42"/>
+      <c r="V3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="W3" s="42"/>
+      <c r="Y3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z3" s="42"/>
+      <c r="AB3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC3" s="42"/>
+      <c r="AE3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="AF3" s="42"/>
+      <c r="AH3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="AI3" s="42"/>
+      <c r="AK3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="AL3" s="42"/>
+      <c r="AN3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="AO3" s="42"/>
+      <c r="AQ3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="AR3" s="42"/>
+      <c r="AT3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="AU3" s="42"/>
     </row>
     <row r="4" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
@@ -2132,6 +2300,50 @@
       <c r="N4" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="S4" s="5"/>
+      <c r="T4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="V4" s="5"/>
+      <c r="W4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="Y4" s="5"/>
+      <c r="Z4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AB4" s="5"/>
+      <c r="AC4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AE4" s="5"/>
+      <c r="AF4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AH4" s="5"/>
+      <c r="AI4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AK4" s="5"/>
+      <c r="AL4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AN4" s="5"/>
+      <c r="AO4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AQ4" s="5"/>
+      <c r="AR4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AT4" s="5"/>
+      <c r="AU4" s="6" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="5" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
@@ -2156,6 +2368,50 @@
       </c>
       <c r="M5" s="5"/>
       <c r="N5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="S5" s="5"/>
+      <c r="T5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="V5" s="5"/>
+      <c r="W5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y5" s="5"/>
+      <c r="Z5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB5" s="5"/>
+      <c r="AC5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE5" s="5"/>
+      <c r="AF5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH5" s="5"/>
+      <c r="AI5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AK5" s="5"/>
+      <c r="AL5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AN5" s="5"/>
+      <c r="AO5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AQ5" s="5"/>
+      <c r="AR5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AT5" s="5"/>
+      <c r="AU5" s="6" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2195,6 +2451,83 @@
       <c r="N6" s="6" t="s">
         <v>4</v>
       </c>
+      <c r="P6" s="5">
+        <f>SUM(P4+P5)</f>
+        <v>0</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="S6" s="5">
+        <f>SUM(S4+S5)</f>
+        <v>0</v>
+      </c>
+      <c r="T6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="V6" s="5">
+        <f>SUM(V4+V5)</f>
+        <v>0</v>
+      </c>
+      <c r="W6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="Y6" s="5">
+        <f>SUM(Y4+Y5)</f>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AB6" s="5">
+        <f>SUM(AB4+AB5)</f>
+        <v>0</v>
+      </c>
+      <c r="AC6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AE6" s="5">
+        <f>SUM(AE4+AE5)</f>
+        <v>0</v>
+      </c>
+      <c r="AF6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH6" s="5">
+        <f>SUM(AH4+AH5)</f>
+        <v>0</v>
+      </c>
+      <c r="AI6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AK6" s="5">
+        <f>SUM(AK4+AK5)</f>
+        <v>0</v>
+      </c>
+      <c r="AL6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AN6" s="5">
+        <f>SUM(AN4+AN5)</f>
+        <v>0</v>
+      </c>
+      <c r="AO6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AQ6" s="5">
+        <f>SUM(AQ4+AQ5)</f>
+        <v>0</v>
+      </c>
+      <c r="AR6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AT6" s="5">
+        <f>SUM(AT4+AT5)</f>
+        <v>0</v>
+      </c>
+      <c r="AU6" s="6" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="7" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
@@ -2220,6 +2553,50 @@
         <v>5</v>
       </c>
       <c r="N8" s="43"/>
+      <c r="P8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q8" s="43"/>
+      <c r="S8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="T8" s="43"/>
+      <c r="V8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="W8" s="43"/>
+      <c r="Y8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="Z8" s="43"/>
+      <c r="AB8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="AC8" s="43"/>
+      <c r="AE8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="AF8" s="43"/>
+      <c r="AH8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="AI8" s="43"/>
+      <c r="AK8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="AL8" s="43"/>
+      <c r="AN8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="AO8" s="43"/>
+      <c r="AQ8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="AR8" s="43"/>
+      <c r="AT8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="AU8" s="43"/>
     </row>
     <row r="9" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
@@ -2246,6 +2623,50 @@
       <c r="N9" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="S9" s="5"/>
+      <c r="T9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="V9" s="5"/>
+      <c r="W9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="Y9" s="5"/>
+      <c r="Z9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AB9" s="5"/>
+      <c r="AC9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AE9" s="5"/>
+      <c r="AF9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AH9" s="5"/>
+      <c r="AI9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AK9" s="5"/>
+      <c r="AL9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AN9" s="5"/>
+      <c r="AO9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AQ9" s="5"/>
+      <c r="AR9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AT9" s="5"/>
+      <c r="AU9" s="6" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
@@ -2270,6 +2691,50 @@
       </c>
       <c r="M10" s="5"/>
       <c r="N10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="S10" s="5"/>
+      <c r="T10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="V10" s="5"/>
+      <c r="W10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y10" s="5"/>
+      <c r="Z10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB10" s="5"/>
+      <c r="AC10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE10" s="5"/>
+      <c r="AF10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH10" s="5"/>
+      <c r="AI10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AK10" s="5"/>
+      <c r="AL10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AN10" s="5"/>
+      <c r="AO10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AQ10" s="5"/>
+      <c r="AR10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="AT10" s="5"/>
+      <c r="AU10" s="6" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2309,6 +2774,83 @@
       <c r="N11" s="6" t="s">
         <v>4</v>
       </c>
+      <c r="P11" s="5">
+        <f>SUM(P9+P10)</f>
+        <v>0</v>
+      </c>
+      <c r="Q11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="S11" s="5">
+        <f>SUM(S9+S10)</f>
+        <v>0</v>
+      </c>
+      <c r="T11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="V11" s="5">
+        <f>SUM(V9+V10)</f>
+        <v>0</v>
+      </c>
+      <c r="W11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="Y11" s="5">
+        <f>SUM(Y9+Y10)</f>
+        <v>0</v>
+      </c>
+      <c r="Z11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AB11" s="5">
+        <f>SUM(AB9+AB10)</f>
+        <v>0</v>
+      </c>
+      <c r="AC11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AE11" s="5">
+        <f>SUM(AE9+AE10)</f>
+        <v>0</v>
+      </c>
+      <c r="AF11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH11" s="5">
+        <f>SUM(AH9+AH10)</f>
+        <v>0</v>
+      </c>
+      <c r="AI11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AK11" s="5">
+        <f>SUM(AK9+AK10)</f>
+        <v>0</v>
+      </c>
+      <c r="AL11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AN11" s="5">
+        <f>SUM(AN9+AN10)</f>
+        <v>0</v>
+      </c>
+      <c r="AO11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AQ11" s="5">
+        <f>SUM(AQ9+AQ10)</f>
+        <v>0</v>
+      </c>
+      <c r="AR11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AT11" s="5">
+        <f>SUM(AT9+AT10)</f>
+        <v>0</v>
+      </c>
+      <c r="AU11" s="6" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="12" x14ac:dyDescent="0.25">
       <c r="D12" s="3"/>
@@ -2334,6 +2876,50 @@
         <v>6</v>
       </c>
       <c r="N13" s="44"/>
+      <c r="P13" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q13" s="44"/>
+      <c r="S13" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="T13" s="44"/>
+      <c r="V13" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="W13" s="44"/>
+      <c r="Y13" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="Z13" s="44"/>
+      <c r="AB13" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC13" s="44"/>
+      <c r="AE13" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="AF13" s="44"/>
+      <c r="AH13" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI13" s="44"/>
+      <c r="AK13" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="AL13" s="44"/>
+      <c r="AN13" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="AO13" s="44"/>
+      <c r="AQ13" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="AR13" s="44"/>
+      <c r="AT13" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="AU13" s="44"/>
     </row>
     <row r="14" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
@@ -2371,6 +2957,83 @@
       <c r="N14" s="6" t="s">
         <v>7</v>
       </c>
+      <c r="P14" s="5">
+        <f>SUM(P6+P11)</f>
+        <v>0</v>
+      </c>
+      <c r="Q14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="S14" s="5">
+        <f>SUM(S6+S11)</f>
+        <v>0</v>
+      </c>
+      <c r="T14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="V14" s="5">
+        <f>SUM(V6+V11)</f>
+        <v>0</v>
+      </c>
+      <c r="W14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="Y14" s="5">
+        <f>SUM(Y6+Y11)</f>
+        <v>0</v>
+      </c>
+      <c r="Z14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="AB14" s="5">
+        <f>SUM(AB6+AB11)</f>
+        <v>0</v>
+      </c>
+      <c r="AC14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="AE14" s="5">
+        <f>SUM(AE6+AE11)</f>
+        <v>0</v>
+      </c>
+      <c r="AF14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="AH14" s="5">
+        <f>SUM(AH6+AH11)</f>
+        <v>0</v>
+      </c>
+      <c r="AI14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="AK14" s="5">
+        <f>SUM(AK6+AK11)</f>
+        <v>0</v>
+      </c>
+      <c r="AL14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="AN14" s="5">
+        <f>SUM(AN6+AN11)</f>
+        <v>0</v>
+      </c>
+      <c r="AO14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="AQ14" s="5">
+        <f>SUM(AQ6+AQ11)</f>
+        <v>0</v>
+      </c>
+      <c r="AR14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="AT14" s="5">
+        <f>SUM(AT6+AT11)</f>
+        <v>0</v>
+      </c>
+      <c r="AU14" s="6" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="15" x14ac:dyDescent="0.25">
       <c r="D15" s="3"/>
@@ -2378,19 +3041,19 @@
     <row r="16">
       <c r="A16" s="31" t="inlineStr">
         <is>
-          <t>Yellow cells = type this week's numbers here, from Aptean EAM &gt; Open Work Orders: the date, then repair tickets and PMs for each plant.</t>
+          <t>Yellow cells = type this week's numbers here, from Aptean EAM &gt; Open Work Orders: repair tickets and PMs for each plant. A block only counts once it has numbers.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="31" t="inlineStr">
         <is>
-          <t>When the empty blocks are used up: copy the newest block (for example M1:N14), paste it 3 columns to the right (P1), and fill in the yellow cells. The chart on Sheet1 updates by itself.</t>
+          <t>Blocks are ready through 12/28/2026 (the date on each is the Monday; change it if you pull on another day). After that: copy the newest block (for example AT1:AU14), paste it 3 columns to the right (AW1), type the date and fill in the yellow cells.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="48">
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A13:B13"/>
@@ -2406,6 +3069,39 @@
     <mergeCell ref="M3:N3"/>
     <mergeCell ref="M8:N8"/>
     <mergeCell ref="M13:N13"/>
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="P13:Q13"/>
+    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="S13:T13"/>
+    <mergeCell ref="V3:W3"/>
+    <mergeCell ref="V8:W8"/>
+    <mergeCell ref="V13:W13"/>
+    <mergeCell ref="Y3:Z3"/>
+    <mergeCell ref="Y8:Z8"/>
+    <mergeCell ref="Y13:Z13"/>
+    <mergeCell ref="AB3:AC3"/>
+    <mergeCell ref="AB8:AC8"/>
+    <mergeCell ref="AB13:AC13"/>
+    <mergeCell ref="AE3:AF3"/>
+    <mergeCell ref="AE8:AF8"/>
+    <mergeCell ref="AE13:AF13"/>
+    <mergeCell ref="AH3:AI3"/>
+    <mergeCell ref="AH8:AI8"/>
+    <mergeCell ref="AH13:AI13"/>
+    <mergeCell ref="AK3:AL3"/>
+    <mergeCell ref="AK8:AL8"/>
+    <mergeCell ref="AK13:AL13"/>
+    <mergeCell ref="AN3:AO3"/>
+    <mergeCell ref="AN8:AO8"/>
+    <mergeCell ref="AN13:AO13"/>
+    <mergeCell ref="AQ3:AR3"/>
+    <mergeCell ref="AQ8:AR8"/>
+    <mergeCell ref="AQ13:AR13"/>
+    <mergeCell ref="AT3:AU3"/>
+    <mergeCell ref="AT8:AU8"/>
+    <mergeCell ref="AT13:AU13"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:ZZ1">
     <cfRule type="expression" dxfId="18" priority="1">
@@ -2432,7 +3128,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -2452,7 +3148,7 @@
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="33" t="inlineStr">
         <is>
-          <t>Updates by itself from the Totals page: each dated block there (every 3 columns: A, D, G, J, M ...) is one week.</t>
+          <t>Updates by itself from the Totals page: every block there that has a date and numbers is one week.</t>
         </is>
       </c>
     </row>
@@ -2487,15 +3183,15 @@
     </row>
     <row r="22">
       <c r="A22" s="39">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v>46280</v>
       </c>
       <c r="B22" s="38">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v>11</v>
       </c>
       <c r="C22" s="38">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v>3</v>
       </c>
       <c r="D22" s="40">
@@ -2503,11 +3199,11 @@
         <v>14</v>
       </c>
       <c r="E22" s="38">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v>32</v>
       </c>
       <c r="F22" s="38">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v>173</v>
       </c>
       <c r="G22" s="40">
@@ -2525,15 +3221,15 @@
     </row>
     <row r="23">
       <c r="A23" s="39">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v>46286</v>
       </c>
       <c r="B23" s="38">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v>7</v>
       </c>
       <c r="C23" s="38">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v>6</v>
       </c>
       <c r="D23" s="40">
@@ -2541,11 +3237,11 @@
         <v>13</v>
       </c>
       <c r="E23" s="38">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v>38</v>
       </c>
       <c r="F23" s="38">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v>241</v>
       </c>
       <c r="G23" s="40">
@@ -2563,15 +3259,15 @@
     </row>
     <row r="24">
       <c r="A24" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B24" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C24" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D24" s="40" t="str">
@@ -2579,11 +3275,11 @@
         <v/>
       </c>
       <c r="E24" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F24" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G24" s="40" t="str">
@@ -2601,15 +3297,15 @@
     </row>
     <row r="25">
       <c r="A25" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B25" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C25" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D25" s="40" t="str">
@@ -2617,11 +3313,11 @@
         <v/>
       </c>
       <c r="E25" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F25" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G25" s="40" t="str">
@@ -2639,15 +3335,15 @@
     </row>
     <row r="26">
       <c r="A26" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B26" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C26" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D26" s="40" t="str">
@@ -2655,11 +3351,11 @@
         <v/>
       </c>
       <c r="E26" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F26" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G26" s="40" t="str">
@@ -2677,15 +3373,15 @@
     </row>
     <row r="27">
       <c r="A27" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B27" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C27" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D27" s="40" t="str">
@@ -2693,11 +3389,11 @@
         <v/>
       </c>
       <c r="E27" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F27" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G27" s="40" t="str">
@@ -2715,15 +3411,15 @@
     </row>
     <row r="28">
       <c r="A28" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B28" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C28" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D28" s="40" t="str">
@@ -2731,11 +3427,11 @@
         <v/>
       </c>
       <c r="E28" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F28" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G28" s="40" t="str">
@@ -2753,15 +3449,15 @@
     </row>
     <row r="29">
       <c r="A29" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B29" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C29" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D29" s="40" t="str">
@@ -2769,11 +3465,11 @@
         <v/>
       </c>
       <c r="E29" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F29" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G29" s="40" t="str">
@@ -2791,15 +3487,15 @@
     </row>
     <row r="30">
       <c r="A30" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B30" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C30" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D30" s="40" t="str">
@@ -2807,11 +3503,11 @@
         <v/>
       </c>
       <c r="E30" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F30" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G30" s="40" t="str">
@@ -2829,15 +3525,15 @@
     </row>
     <row r="31">
       <c r="A31" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B31" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C31" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D31" s="40" t="str">
@@ -2845,11 +3541,11 @@
         <v/>
       </c>
       <c r="E31" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F31" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G31" s="40" t="str">
@@ -2867,15 +3563,15 @@
     </row>
     <row r="32">
       <c r="A32" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B32" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C32" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D32" s="40" t="str">
@@ -2883,11 +3579,11 @@
         <v/>
       </c>
       <c r="E32" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F32" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G32" s="40" t="str">
@@ -2905,15 +3601,15 @@
     </row>
     <row r="33">
       <c r="A33" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B33" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C33" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D33" s="40" t="str">
@@ -2921,11 +3617,11 @@
         <v/>
       </c>
       <c r="E33" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F33" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G33" s="40" t="str">
@@ -2943,15 +3639,15 @@
     </row>
     <row r="34">
       <c r="A34" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B34" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C34" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D34" s="40" t="str">
@@ -2959,11 +3655,11 @@
         <v/>
       </c>
       <c r="E34" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F34" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G34" s="40" t="str">
@@ -2981,15 +3677,15 @@
     </row>
     <row r="35">
       <c r="A35" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B35" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C35" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D35" s="40" t="str">
@@ -2997,11 +3693,11 @@
         <v/>
       </c>
       <c r="E35" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F35" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G35" s="40" t="str">
@@ -3019,15 +3715,15 @@
     </row>
     <row r="36">
       <c r="A36" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B36" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C36" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D36" s="40" t="str">
@@ -3035,11 +3731,11 @@
         <v/>
       </c>
       <c r="E36" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F36" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G36" s="40" t="str">
@@ -3057,15 +3753,15 @@
     </row>
     <row r="37">
       <c r="A37" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B37" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C37" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D37" s="40" t="str">
@@ -3073,11 +3769,11 @@
         <v/>
       </c>
       <c r="E37" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F37" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G37" s="40" t="str">
@@ -3095,15 +3791,15 @@
     </row>
     <row r="38">
       <c r="A38" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B38" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C38" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D38" s="40" t="str">
@@ -3111,11 +3807,11 @@
         <v/>
       </c>
       <c r="E38" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F38" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G38" s="40" t="str">
@@ -3133,15 +3829,15 @@
     </row>
     <row r="39">
       <c r="A39" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B39" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C39" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D39" s="40" t="str">
@@ -3149,11 +3845,11 @@
         <v/>
       </c>
       <c r="E39" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F39" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G39" s="40" t="str">
@@ -3171,15 +3867,15 @@
     </row>
     <row r="40">
       <c r="A40" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B40" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C40" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D40" s="40" t="str">
@@ -3187,11 +3883,11 @@
         <v/>
       </c>
       <c r="E40" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F40" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G40" s="40" t="str">
@@ -3209,15 +3905,15 @@
     </row>
     <row r="41">
       <c r="A41" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B41" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C41" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D41" s="40" t="str">
@@ -3225,11 +3921,11 @@
         <v/>
       </c>
       <c r="E41" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F41" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G41" s="40" t="str">
@@ -3247,15 +3943,15 @@
     </row>
     <row r="42">
       <c r="A42" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B42" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C42" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D42" s="40" t="str">
@@ -3263,11 +3959,11 @@
         <v/>
       </c>
       <c r="E42" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F42" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G42" s="40" t="str">
@@ -3285,15 +3981,15 @@
     </row>
     <row r="43">
       <c r="A43" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B43" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C43" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D43" s="40" t="str">
@@ -3301,11 +3997,11 @@
         <v/>
       </c>
       <c r="E43" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F43" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G43" s="40" t="str">
@@ -3323,15 +4019,15 @@
     </row>
     <row r="44">
       <c r="A44" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B44" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C44" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D44" s="40" t="str">
@@ -3339,11 +4035,11 @@
         <v/>
       </c>
       <c r="E44" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F44" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G44" s="40" t="str">
@@ -3361,15 +4057,15 @@
     </row>
     <row r="45">
       <c r="A45" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B45" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C45" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D45" s="40" t="str">
@@ -3377,11 +4073,11 @@
         <v/>
       </c>
       <c r="E45" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F45" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G45" s="40" t="str">
@@ -3399,15 +4095,15 @@
     </row>
     <row r="46">
       <c r="A46" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B46" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C46" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D46" s="40" t="str">
@@ -3415,11 +4111,11 @@
         <v/>
       </c>
       <c r="E46" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F46" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G46" s="40" t="str">
@@ -3437,15 +4133,15 @@
     </row>
     <row r="47">
       <c r="A47" s="39" t="str">
-        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
         <v/>
       </c>
       <c r="B47" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="C47" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="D47" s="40" t="str">
@@ -3453,11 +4149,11 @@
         <v/>
       </c>
       <c r="E47" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="F47" s="38" t="str">
-        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$1:$ZZ$1)/((MOD(COLUMN(Totals!$A$1:$ZZ$1)-2,3)=0)*ISNUMBER(Totals!$A$1:$ZZ$1)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))-1),"")</f>
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
         <v/>
       </c>
       <c r="G47" s="40" t="str">
@@ -3469,6 +4165,538 @@
         <v/>
       </c>
       <c r="I47" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B48" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C48" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D48" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E48" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F48" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G48" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H48" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I48" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B49" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C49" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D49" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E49" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F49" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G49" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H49" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I49" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B50" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C50" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D50" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E50" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F50" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G50" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H50" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I50" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B51" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C51" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D51" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E51" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F51" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G51" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H51" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I51" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B52" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C52" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D52" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E52" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F52" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G52" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H52" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I52" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B53" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C53" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D53" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E53" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F53" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G53" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H53" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I53" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B54" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C54" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D54" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E54" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F54" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G54" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H54" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I54" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B55" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C55" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D55" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E55" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F55" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G55" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H55" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I55" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B56" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C56" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D56" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E56" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F56" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G56" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H56" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I56" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B57" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C57" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D57" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E57" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F57" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G57" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H57" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I57" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B58" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C58" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D58" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E58" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F58" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G58" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H58" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I58" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B59" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C59" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D59" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E59" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F59" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G59" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H59" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I59" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B60" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C60" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D60" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E60" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F60" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G60" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H60" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I60" s="41" t="str">
+        <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="39" t="str">
+        <f>IFERROR(INDEX(Totals!$1:$1,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))+1),"")</f>
+        <v/>
+      </c>
+      <c r="B61" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$4:$4,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="C61" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$5:$5,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="D61" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Repair Tickets]]+WeeklyLog[[#This Row],[Burnsville PMs]])</f>
+        <v/>
+      </c>
+      <c r="E61" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$9:$9,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="F61" s="38" t="str">
+        <f>IFERROR(INDEX(Totals!$10:$10,_xlfn.AGGREGATE(15,6,COLUMN(Totals!$A$4:$ZY$4)/((MOD(COLUMN(Totals!$A$4:$ZY$4)-1,3)=0)*ISNUMBER(Totals!$B$1:$ZZ$1)*((ISNUMBER(Totals!$A$4:$ZY$4)+ISNUMBER(Totals!$A$5:$ZY$5)+ISNUMBER(Totals!$A$9:$ZY$9)+ISNUMBER(Totals!$A$10:$ZY$10))&gt;0)),(ROW()-ROW(WeeklyLog[[#Headers],[Week Of]])))),"")</f>
+        <v/>
+      </c>
+      <c r="G61" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Lakeville Repair Tickets]]+WeeklyLog[[#This Row],[Lakeville PMs]])</f>
+        <v/>
+      </c>
+      <c r="H61" s="40" t="str">
+        <f>IF(WeeklyLog[[#This Row],[Week Of]]="","",WeeklyLog[[#This Row],[Burnsville Total]]+WeeklyLog[[#This Row],[Lakeville Total]])</f>
+        <v/>
+      </c>
+      <c r="I61" s="41" t="str">
         <f ca="1">IFERROR(WeeklyLog[[#This Row],[Combined Total]]-OFFSET(WeeklyLog[[#This Row],[Combined Total]],-1,0),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Rename the chart tab to History and open the tracker on it
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016Ld5yLC3t3yCVGVfyBR5pc
</commit_message>
<xml_diff>
--- a/open-wos-weekly-tracker/Open_WOs_tracker.xlsx
+++ b/open-wos-weekly-tracker/Open_WOs_tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <xr:revisionPtr revIDLastSave="2" documentId="8_{13A66354-4290-446E-B311-AE1A5843A5C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EE88116-21C8-4AA4-8C62-316F6907B512}"/>
   <bookViews>
-    <workbookView activeTab="1" xWindow="285" yWindow="1275" windowWidth="25260" windowHeight="13695" xr2:uid="{C7DEE03B-6693-435C-9B90-2E0F24388ABA}"/>
+    <workbookView activeTab="0" xWindow="285" yWindow="1275" windowWidth="25260" windowHeight="13695" xr2:uid="{C7DEE03B-6693-435C-9B90-2E0F24388ABA}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="17" r:id="rId2"/>
+    <sheet name="History" sheetId="17" r:id="rId2"/>
     <sheet name="Totals" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
@@ -16,9 +16,9 @@
     <definedName name="chart_BV" localSheetId="0">INDEX(WeeklyLog[Burnsville Total],1):INDEX(WeeklyLog[Burnsville Total],MAX(1,COUNT(WeeklyLog[Week Of])))</definedName>
     <definedName name="chart_LV" localSheetId="0">INDEX(WeeklyLog[Lakeville Total],1):INDEX(WeeklyLog[Lakeville Total],MAX(1,COUNT(WeeklyLog[Week Of])))</definedName>
     <definedName name="chart_CO" localSheetId="0">INDEX(WeeklyLog[Combined Total],1):INDEX(WeeklyLog[Combined Total],MAX(1,COUNT(WeeklyLog[Week Of])))</definedName>
-    <definedName name="last_BV" localSheetId="0">IF(Sheet1!chart_Week=MAX(Sheet1!chart_Week),Sheet1!chart_BV,NA())</definedName>
-    <definedName name="last_LV" localSheetId="0">IF(Sheet1!chart_Week=MAX(Sheet1!chart_Week),Sheet1!chart_LV,NA())</definedName>
-    <definedName name="last_CO" localSheetId="0">IF(Sheet1!chart_Week=MAX(Sheet1!chart_Week),Sheet1!chart_CO,NA())</definedName>
+    <definedName name="last_BV" localSheetId="0">IF(History!chart_Week=MAX(History!chart_Week),History!chart_BV,NA())</definedName>
+    <definedName name="last_LV" localSheetId="0">IF(History!chart_Week=MAX(History!chart_Week),History!chart_LV,NA())</definedName>
+    <definedName name="last_CO" localSheetId="0">IF(History!chart_Week=MAX(History!chart_Week),History!chart_CO,NA())</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -983,7 +983,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!chart_Week</c:f>
+              <c:f>History!chart_Week</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
                 <c:ptCount val="2"/>
@@ -998,7 +998,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!chart_BV</c:f>
+              <c:f>History!chart_BV</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1048,7 +1048,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!chart_Week</c:f>
+              <c:f>History!chart_Week</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1063,7 +1063,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!chart_LV</c:f>
+              <c:f>History!chart_LV</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1113,7 +1113,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!chart_Week</c:f>
+              <c:f>History!chart_Week</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1128,7 +1128,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!chart_CO</c:f>
+              <c:f>History!chart_CO</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1201,7 +1201,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!chart_Week</c:f>
+              <c:f>History!chart_Week</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1216,7 +1216,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!last_BV</c:f>
+              <c:f>History!last_BV</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1286,7 +1286,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!chart_Week</c:f>
+              <c:f>History!chart_Week</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1301,7 +1301,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!last_LV</c:f>
+              <c:f>History!last_LV</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1373,7 +1373,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!chart_Week</c:f>
+              <c:f>History!chart_Week</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1388,7 +1388,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!last_CO</c:f>
+              <c:f>History!last_CO</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="2"/>

</xml_diff>